<commit_message>
feat: add the attack vs defense mechanism
</commit_message>
<xml_diff>
--- a/public/gameplay.xlsx
+++ b/public/gameplay.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Uleth\Thesis\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Research\MVC-ARENA\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E39A6F7C-EC7B-4CA5-A83A-DEDE58DF8130}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{391D0398-5A20-4C87-A874-FAC271DB30FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1900" yWindow="920" windowWidth="14400" windowHeight="9160" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="component" sheetId="1" r:id="rId1"/>
@@ -192,7 +192,7 @@
     <t>File Storage Adapter</t>
   </si>
   <si>
-    <t>Authentication and authorization, 2fa</t>
+    <t>Authentication and authorization</t>
   </si>
 </sst>
 </file>
@@ -832,6 +832,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -984,7 +985,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="8" spans="1:4" ht="96.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:4" ht="32.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A8" s="4" t="s">
         <v>4</v>
       </c>
@@ -998,6 +999,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -1053,7 +1055,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="32.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3" ht="16.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A5" s="4" t="s">
         <v>38</v>
       </c>
@@ -1062,7 +1064,7 @@
       </c>
       <c r="C5" s="5"/>
     </row>
-    <row r="6" spans="1:3" ht="48.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3" ht="16.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A6" s="4" t="s">
         <v>40</v>
       </c>
@@ -1071,7 +1073,7 @@
       </c>
       <c r="C6" s="5"/>
     </row>
-    <row r="7" spans="1:3" ht="144.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:3" ht="48.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A7" s="4" t="s">
         <v>41</v>
       </c>

</xml_diff>